<commit_message>
≡ƒÜÇ PO Status update via batch
</commit_message>
<xml_diff>
--- a/po-status.xlsx
+++ b/po-status.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://mvtstechnologies-my.sharepoint.com/personal/edsel_solon_bsegroup_com/Documents/Github Projects/PO_Status/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="2" documentId="11_BEA61AB913BD779C031AE933BD3190EA71D9FE0D" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{FD7D6D67-BEDE-49CD-9B9E-0FC8126ACC79}"/>
+  <xr:revisionPtr revIDLastSave="2" documentId="11_BEA61AB97B2DF2FF0DF8FC911D328CA470D9F83A" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F324E533-6898-4B6F-BA4D-5F01C139A9EF}"/>
   <bookViews>
     <workbookView xWindow="-93" yWindow="-93" windowWidth="25786" windowHeight="13986" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -16,14 +16,14 @@
     <sheet name="PO_StatusQry" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="PO_StatusQry">PO_StatusQry!$A$2:$M$125</definedName>
+    <definedName name="PO_StatusQry">PO_StatusQry!$A$2:$M$127</definedName>
   </definedNames>
   <calcPr calcId="125725"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="379" uniqueCount="203">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="381" uniqueCount="202">
   <si>
     <t>CustName</t>
   </si>
@@ -70,7 +70,7 @@
     <t>4516351202_ASEWH</t>
   </si>
   <si>
-    <t>OverDue by 340 days</t>
+    <t>OverDue by 360 days</t>
   </si>
   <si>
     <t>Texas Instruments SCT</t>
@@ -79,9 +79,6 @@
     <t>4516351202_SCT</t>
   </si>
   <si>
-    <t>Varies (2025-08-29 → 2026-07-28)</t>
-  </si>
-  <si>
     <t>Texas Instruments Taiwan</t>
   </si>
   <si>
@@ -103,7 +100,250 @@
     <t>Global PO 4516351202</t>
   </si>
   <si>
-    <t>OverDue by 176 days</t>
+    <t>OverDue by 196 days</t>
+  </si>
+  <si>
+    <t>Analog Devices Gen. Trias Inc. (ADGT)</t>
+  </si>
+  <si>
+    <t>47270551</t>
+  </si>
+  <si>
+    <t>OverDue by 119 days</t>
+  </si>
+  <si>
+    <t>47318424</t>
+  </si>
+  <si>
+    <t>OverDue by 103 days</t>
+  </si>
+  <si>
+    <t>Varies (2026-05-13 → 2026-09-01)</t>
+  </si>
+  <si>
+    <t>ASE CO., LTD - PHILIPPINES BRANCH 01-075</t>
+  </si>
+  <si>
+    <t>MO262002496</t>
+  </si>
+  <si>
+    <t>OverDue by 70 days</t>
+  </si>
+  <si>
+    <t>UTAC Thai Limited ( UTL 3)</t>
+  </si>
+  <si>
+    <t>PO-468-061326-01</t>
+  </si>
+  <si>
+    <t>OverDue by 32 days</t>
+  </si>
+  <si>
+    <t>Tongfu Microelectronics Co.,Ltd.</t>
+  </si>
+  <si>
+    <t>4516351202_NFME</t>
+  </si>
+  <si>
+    <t>OverDue by 27 days</t>
+  </si>
+  <si>
+    <t>47301012</t>
+  </si>
+  <si>
+    <t>17 days before Due</t>
+  </si>
+  <si>
+    <t>TI (Philippines) Inc.</t>
+  </si>
+  <si>
+    <t>4516351202_TIPI</t>
+  </si>
+  <si>
+    <t>3 days before Due</t>
+  </si>
+  <si>
+    <t>NXP Malaysia Sdn. Bhd.</t>
+  </si>
+  <si>
+    <t>3T/PO262347</t>
+  </si>
+  <si>
+    <t>2 days before Due</t>
+  </si>
+  <si>
+    <t>3T/PO262348</t>
+  </si>
+  <si>
+    <t>Texas Instruments Japan Limited MIHO Plant (MIHO 8 FAB)</t>
+  </si>
+  <si>
+    <t>4516351202_MIHO</t>
+  </si>
+  <si>
+    <t>1 days before Due</t>
+  </si>
+  <si>
+    <t>Texas Instruments AIZU</t>
+  </si>
+  <si>
+    <t>4516351202_AIZU</t>
+  </si>
+  <si>
+    <t>Due Today</t>
+  </si>
+  <si>
+    <t>TEXAS INSTRUMENTS (INDIA) Pvt. Ltd</t>
+  </si>
+  <si>
+    <t>4516351202_TII</t>
+  </si>
+  <si>
+    <t>TBA_NXP</t>
+  </si>
+  <si>
+    <t>Hana Semiconductor (Ayutthaya) Co., Ltd (HNT)</t>
+  </si>
+  <si>
+    <t>4516351202_HNT</t>
+  </si>
+  <si>
+    <t>4516351202_UTL</t>
+  </si>
+  <si>
+    <t>Lingsen Precision Industries Ltd.</t>
+  </si>
+  <si>
+    <t>4516446856</t>
+  </si>
+  <si>
+    <t>Texas Instruments DMOS5</t>
+  </si>
+  <si>
+    <t>4516351202_DMOS5</t>
+  </si>
+  <si>
+    <t>Texas Instruments LFAB</t>
+  </si>
+  <si>
+    <t>4516351202_LFAB</t>
+  </si>
+  <si>
+    <t>Texas Instruments Taiwan Limited</t>
+  </si>
+  <si>
+    <t>4516450237</t>
+  </si>
+  <si>
+    <t>ANALOG DEVICES INC.</t>
+  </si>
+  <si>
+    <t>47369322</t>
+  </si>
+  <si>
+    <t>ROCHESTER ELECTRONICS</t>
+  </si>
+  <si>
+    <t>252395</t>
+  </si>
+  <si>
+    <t>47188646</t>
+  </si>
+  <si>
+    <t>Completed PO</t>
+  </si>
+  <si>
+    <t>47218149</t>
+  </si>
+  <si>
+    <t>47245848</t>
+  </si>
+  <si>
+    <t>47245933</t>
+  </si>
+  <si>
+    <t>47253728</t>
+  </si>
+  <si>
+    <t>47264622</t>
+  </si>
+  <si>
+    <t>47274630</t>
+  </si>
+  <si>
+    <t>47276474</t>
+  </si>
+  <si>
+    <t>47283634</t>
+  </si>
+  <si>
+    <t>47283654</t>
+  </si>
+  <si>
+    <t>47286185</t>
+  </si>
+  <si>
+    <t>47289023</t>
+  </si>
+  <si>
+    <t>47290167</t>
+  </si>
+  <si>
+    <t>47292239</t>
+  </si>
+  <si>
+    <t>47292914</t>
+  </si>
+  <si>
+    <t>47296581</t>
+  </si>
+  <si>
+    <t>47296806</t>
+  </si>
+  <si>
+    <t>47301646</t>
+  </si>
+  <si>
+    <t>47304169</t>
+  </si>
+  <si>
+    <t>47324752</t>
+  </si>
+  <si>
+    <t>47345978</t>
+  </si>
+  <si>
+    <t>47352135</t>
+  </si>
+  <si>
+    <t>47361598</t>
+  </si>
+  <si>
+    <t>47361669</t>
+  </si>
+  <si>
+    <t>47362207</t>
+  </si>
+  <si>
+    <t>47362715</t>
+  </si>
+  <si>
+    <t>47364135</t>
+  </si>
+  <si>
+    <t>47375825</t>
+  </si>
+  <si>
+    <t>TBA_ADGT</t>
+  </si>
+  <si>
+    <t>TBD_SAMPLE</t>
+  </si>
+  <si>
+    <t>ANALOG DEVICES INC. CAMAS</t>
+  </si>
+  <si>
+    <t>47259467</t>
   </si>
   <si>
     <t>ARDENTEC CORPORATION</t>
@@ -112,271 +352,37 @@
     <t>4516351202_ARD</t>
   </si>
   <si>
-    <t>OverDue by 130 days</t>
-  </si>
-  <si>
-    <t>Varies (2026-03-27 → 2026-05-19)</t>
-  </si>
-  <si>
-    <t>Analog Devices Gen. Trias Inc. (ADGT)</t>
-  </si>
-  <si>
-    <t>47270551</t>
-  </si>
-  <si>
-    <t>OverDue by 99 days</t>
-  </si>
-  <si>
-    <t>TI (Philippines) Inc.</t>
-  </si>
-  <si>
-    <t>4516351202_TIPI</t>
-  </si>
-  <si>
-    <t>Varies (2026-04-27 → 2026-06-25)</t>
-  </si>
-  <si>
-    <t>47318424</t>
-  </si>
-  <si>
-    <t>OverDue by 83 days</t>
-  </si>
-  <si>
-    <t>Varies (2026-05-13 → 2026-08-25)</t>
-  </si>
-  <si>
-    <t>ASE CO., LTD - PHILIPPINES BRANCH 01-075</t>
-  </si>
-  <si>
-    <t>MO262002496</t>
-  </si>
-  <si>
-    <t>OverDue by 50 days</t>
-  </si>
-  <si>
-    <t>UTAC Thai Limited ( UTL 3)</t>
-  </si>
-  <si>
-    <t>PO-468-061326-01</t>
-  </si>
-  <si>
-    <t>OverDue by 12 days</t>
-  </si>
-  <si>
-    <t>Tongfu Microelectronics Co.,Ltd.</t>
-  </si>
-  <si>
-    <t>4516351202_NFME</t>
-  </si>
-  <si>
-    <t>OverDue by 7 days</t>
+    <t>Ardentec Korea Co., Ltd.</t>
+  </si>
+  <si>
+    <t>4516351202_ATK</t>
+  </si>
+  <si>
+    <t>ATX SEMICONDUCTOR (SHANGHAI) CO.,LTD.</t>
+  </si>
+  <si>
+    <t>4516351202_ASESH</t>
   </si>
   <si>
     <t>AVAGO TECHNOLOGIES_x000D_
 INTERNATIONAL SALES PTE LTD</t>
   </si>
   <si>
+    <t>8541541216</t>
+  </si>
+  <si>
+    <t>8541550629</t>
+  </si>
+  <si>
+    <t>8541550824</t>
+  </si>
+  <si>
+    <t>8541563942</t>
+  </si>
+  <si>
     <t>8541571063</t>
   </si>
   <si>
-    <t>OverDue by 6 days</t>
-  </si>
-  <si>
-    <t>47364135</t>
-  </si>
-  <si>
-    <t>14 days before Due</t>
-  </si>
-  <si>
-    <t>Texas Instruments AIZU</t>
-  </si>
-  <si>
-    <t>4516351202_AIZU</t>
-  </si>
-  <si>
-    <t>9 days before Due</t>
-  </si>
-  <si>
-    <t>NXP Malaysia Sdn. Bhd.</t>
-  </si>
-  <si>
-    <t>TBA_NXP</t>
-  </si>
-  <si>
-    <t>6 days before Due</t>
-  </si>
-  <si>
-    <t>TEXAS INSTRUMENTS (INDIA) Pvt. Ltd</t>
-  </si>
-  <si>
-    <t>4516351202_TII</t>
-  </si>
-  <si>
-    <t>3T/PO262348</t>
-  </si>
-  <si>
-    <t>Texas Instruments Taiwan Limited</t>
-  </si>
-  <si>
-    <t>4516450237</t>
-  </si>
-  <si>
-    <t>3T/PO262347</t>
-  </si>
-  <si>
-    <t>4516351202_UTL</t>
-  </si>
-  <si>
-    <t>Texas Instruments DMOS5</t>
-  </si>
-  <si>
-    <t>4516351202_DMOS5</t>
-  </si>
-  <si>
-    <t>Texas Instruments LFAB</t>
-  </si>
-  <si>
-    <t>4516351202_LFAB</t>
-  </si>
-  <si>
-    <t>ANALOG DEVICES INC.</t>
-  </si>
-  <si>
-    <t>47369322</t>
-  </si>
-  <si>
-    <t>ROCHESTER ELECTRONICS</t>
-  </si>
-  <si>
-    <t>252395</t>
-  </si>
-  <si>
-    <t>Texas Instruments Japan Limited MIHO Plant (MIHO 8 FAB)</t>
-  </si>
-  <si>
-    <t>4516351202_MIHO</t>
-  </si>
-  <si>
-    <t>Completed PO</t>
-  </si>
-  <si>
-    <t>47188646</t>
-  </si>
-  <si>
-    <t>47218149</t>
-  </si>
-  <si>
-    <t>47245848</t>
-  </si>
-  <si>
-    <t>47245933</t>
-  </si>
-  <si>
-    <t>47253728</t>
-  </si>
-  <si>
-    <t>47264622</t>
-  </si>
-  <si>
-    <t>47274630</t>
-  </si>
-  <si>
-    <t>47276474</t>
-  </si>
-  <si>
-    <t>47283634</t>
-  </si>
-  <si>
-    <t>47283654</t>
-  </si>
-  <si>
-    <t>47286185</t>
-  </si>
-  <si>
-    <t>47289023</t>
-  </si>
-  <si>
-    <t>47290167</t>
-  </si>
-  <si>
-    <t>47292239</t>
-  </si>
-  <si>
-    <t>47292914</t>
-  </si>
-  <si>
-    <t>47296581</t>
-  </si>
-  <si>
-    <t>47296806</t>
-  </si>
-  <si>
-    <t>47301012</t>
-  </si>
-  <si>
-    <t>47301646</t>
-  </si>
-  <si>
-    <t>47304169</t>
-  </si>
-  <si>
-    <t>47324752</t>
-  </si>
-  <si>
-    <t>47345978</t>
-  </si>
-  <si>
-    <t>47352135</t>
-  </si>
-  <si>
-    <t>47361598</t>
-  </si>
-  <si>
-    <t>47361669</t>
-  </si>
-  <si>
-    <t>47362207</t>
-  </si>
-  <si>
-    <t>47362715</t>
-  </si>
-  <si>
-    <t>TBA_ADGT</t>
-  </si>
-  <si>
-    <t>TBD_SAMPLE</t>
-  </si>
-  <si>
-    <t>ANALOG DEVICES INC. CAMAS</t>
-  </si>
-  <si>
-    <t>47259467</t>
-  </si>
-  <si>
-    <t>Ardentec Korea Co., Ltd.</t>
-  </si>
-  <si>
-    <t>4516351202_ATK</t>
-  </si>
-  <si>
-    <t>ATX SEMICONDUCTOR (SHANGHAI) CO.,LTD.</t>
-  </si>
-  <si>
-    <t>4516351202_ASESH</t>
-  </si>
-  <si>
-    <t>8541541216</t>
-  </si>
-  <si>
-    <t>8541550629</t>
-  </si>
-  <si>
-    <t>8541550824</t>
-  </si>
-  <si>
-    <t>8541563942</t>
-  </si>
-  <si>
     <t>Boston Semi Equipment</t>
   </si>
   <si>
@@ -425,12 +431,6 @@
     <t>TBD_EVALUATION</t>
   </si>
   <si>
-    <t>Hana Semiconductor (Ayutthaya) Co., Ltd (HNT)</t>
-  </si>
-  <si>
-    <t>4516351202_HNT</t>
-  </si>
-  <si>
     <t>4910172298</t>
   </si>
   <si>
@@ -440,15 +440,9 @@
     <t>ES072525</t>
   </si>
   <si>
-    <t>Lingsen Precision Industries Ltd.</t>
-  </si>
-  <si>
     <t>4516260169</t>
   </si>
   <si>
-    <t>4516446856</t>
-  </si>
-  <si>
     <t>LPI-2507174</t>
   </si>
   <si>
@@ -632,7 +626,10 @@
     <t>43156228</t>
   </si>
   <si>
-    <t>Last updated: 2026-08-04 14:04:31</t>
+    <t>PO002810</t>
+  </si>
+  <si>
+    <t>Last updated: 2026-08-24 08:41:10</t>
   </si>
 </sst>
 </file>
@@ -977,12 +974,12 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:M125"/>
+  <dimension ref="A1:M127"/>
   <sheetFormatPr defaultRowHeight="14.35" x14ac:dyDescent="0.5"/>
   <sheetData>
     <row r="1" spans="1:13" x14ac:dyDescent="0.5">
       <c r="A1" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
     </row>
     <row r="2" spans="1:13" x14ac:dyDescent="0.5">
@@ -1055,7 +1052,7 @@
         <v>45898</v>
       </c>
       <c r="K3">
-        <v>-340</v>
+        <v>-360</v>
       </c>
       <c r="L3" t="s">
         <v>15</v>
@@ -1072,42 +1069,39 @@
         <v>355</v>
       </c>
       <c r="D4">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E4">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F4">
-        <v>11</v>
+        <v>0</v>
       </c>
       <c r="H4">
-        <v>339</v>
+        <v>351</v>
       </c>
       <c r="I4">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J4" s="1">
         <v>45898</v>
       </c>
       <c r="K4">
-        <v>-340</v>
+        <v>-360</v>
       </c>
       <c r="L4" t="s">
         <v>15</v>
       </c>
-      <c r="M4" t="s">
-        <v>18</v>
-      </c>
     </row>
     <row r="5" spans="1:13" x14ac:dyDescent="0.5">
       <c r="A5" t="s">
+        <v>18</v>
+      </c>
+      <c r="B5" t="s">
         <v>19</v>
       </c>
-      <c r="B5" t="s">
-        <v>20</v>
-      </c>
       <c r="C5">
-        <v>269</v>
+        <v>272</v>
       </c>
       <c r="D5">
         <v>0</v>
@@ -1116,7 +1110,7 @@
         <v>2</v>
       </c>
       <c r="F5">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="H5">
         <v>266</v>
@@ -1128,7 +1122,7 @@
         <v>45898</v>
       </c>
       <c r="K5">
-        <v>-340</v>
+        <v>-360</v>
       </c>
       <c r="L5" t="s">
         <v>15</v>
@@ -1136,25 +1130,25 @@
     </row>
     <row r="6" spans="1:13" x14ac:dyDescent="0.5">
       <c r="A6" t="s">
+        <v>20</v>
+      </c>
+      <c r="B6" t="s">
         <v>21</v>
       </c>
-      <c r="B6" t="s">
-        <v>22</v>
-      </c>
       <c r="C6">
-        <v>222</v>
+        <v>226</v>
       </c>
       <c r="D6">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="E6">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="F6">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="H6">
-        <v>199</v>
+        <v>205</v>
       </c>
       <c r="I6">
         <v>0</v>
@@ -1163,24 +1157,24 @@
         <v>45898</v>
       </c>
       <c r="K6">
-        <v>-340</v>
+        <v>-360</v>
       </c>
       <c r="L6" t="s">
         <v>15</v>
       </c>
       <c r="M6" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
     <row r="7" spans="1:13" x14ac:dyDescent="0.5">
       <c r="A7" t="s">
+        <v>23</v>
+      </c>
+      <c r="B7" t="s">
         <v>24</v>
       </c>
-      <c r="B7" t="s">
-        <v>25</v>
-      </c>
       <c r="C7">
-        <v>207</v>
+        <v>217</v>
       </c>
       <c r="D7">
         <v>0</v>
@@ -1189,220 +1183,214 @@
         <v>1</v>
       </c>
       <c r="F7">
-        <v>11</v>
+        <v>1</v>
       </c>
       <c r="H7">
-        <v>195</v>
+        <v>213</v>
       </c>
       <c r="I7">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="J7" s="1">
         <v>46062</v>
       </c>
       <c r="K7">
-        <v>-176</v>
+        <v>-196</v>
       </c>
       <c r="L7" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
     </row>
     <row r="8" spans="1:13" x14ac:dyDescent="0.5">
       <c r="A8" t="s">
+        <v>26</v>
+      </c>
+      <c r="B8" t="s">
         <v>27</v>
       </c>
-      <c r="B8" t="s">
+      <c r="C8">
+        <v>29</v>
+      </c>
+      <c r="D8">
+        <v>0</v>
+      </c>
+      <c r="E8">
+        <v>2</v>
+      </c>
+      <c r="F8">
+        <v>0</v>
+      </c>
+      <c r="H8">
+        <v>27</v>
+      </c>
+      <c r="I8">
+        <v>0</v>
+      </c>
+      <c r="J8" s="1">
+        <v>46139</v>
+      </c>
+      <c r="K8">
+        <v>-119</v>
+      </c>
+      <c r="L8" t="s">
         <v>28</v>
-      </c>
-      <c r="C8">
-        <v>259</v>
-      </c>
-      <c r="D8">
-        <v>1</v>
-      </c>
-      <c r="E8">
-        <v>5</v>
-      </c>
-      <c r="F8">
-        <v>0</v>
-      </c>
-      <c r="H8">
-        <v>253</v>
-      </c>
-      <c r="I8">
-        <v>0</v>
-      </c>
-      <c r="J8" s="1">
-        <v>46108</v>
-      </c>
-      <c r="K8">
-        <v>-130</v>
-      </c>
-      <c r="L8" t="s">
-        <v>29</v>
-      </c>
-      <c r="M8" t="s">
-        <v>30</v>
       </c>
     </row>
     <row r="9" spans="1:13" x14ac:dyDescent="0.5">
       <c r="A9" t="s">
+        <v>26</v>
+      </c>
+      <c r="B9" t="s">
+        <v>29</v>
+      </c>
+      <c r="C9">
+        <v>41</v>
+      </c>
+      <c r="D9">
+        <v>1</v>
+      </c>
+      <c r="E9">
+        <v>21</v>
+      </c>
+      <c r="F9">
+        <v>0</v>
+      </c>
+      <c r="H9">
+        <v>19</v>
+      </c>
+      <c r="I9">
+        <v>0</v>
+      </c>
+      <c r="J9" s="1">
+        <v>46155</v>
+      </c>
+      <c r="K9">
+        <v>-103</v>
+      </c>
+      <c r="L9" t="s">
+        <v>30</v>
+      </c>
+      <c r="M9" t="s">
         <v>31</v>
-      </c>
-      <c r="B9" t="s">
-        <v>32</v>
-      </c>
-      <c r="C9">
-        <v>29</v>
-      </c>
-      <c r="D9">
-        <v>0</v>
-      </c>
-      <c r="E9">
-        <v>2</v>
-      </c>
-      <c r="F9">
-        <v>0</v>
-      </c>
-      <c r="H9">
-        <v>27</v>
-      </c>
-      <c r="I9">
-        <v>0</v>
-      </c>
-      <c r="J9" s="1">
-        <v>46139</v>
-      </c>
-      <c r="K9">
-        <v>-99</v>
-      </c>
-      <c r="L9" t="s">
-        <v>33</v>
       </c>
     </row>
     <row r="10" spans="1:13" x14ac:dyDescent="0.5">
       <c r="A10" t="s">
+        <v>32</v>
+      </c>
+      <c r="B10" t="s">
+        <v>33</v>
+      </c>
+      <c r="C10">
+        <v>1</v>
+      </c>
+      <c r="D10">
+        <v>0</v>
+      </c>
+      <c r="E10">
+        <v>1</v>
+      </c>
+      <c r="F10">
+        <v>0</v>
+      </c>
+      <c r="H10">
+        <v>0</v>
+      </c>
+      <c r="I10">
+        <v>0</v>
+      </c>
+      <c r="J10" s="1">
+        <v>46188</v>
+      </c>
+      <c r="K10">
+        <v>-70</v>
+      </c>
+      <c r="L10" t="s">
         <v>34</v>
-      </c>
-      <c r="B10" t="s">
-        <v>35</v>
-      </c>
-      <c r="C10">
-        <v>666</v>
-      </c>
-      <c r="D10">
-        <v>0</v>
-      </c>
-      <c r="E10">
-        <v>3</v>
-      </c>
-      <c r="F10">
-        <v>20</v>
-      </c>
-      <c r="H10">
-        <v>643</v>
-      </c>
-      <c r="I10">
-        <v>0</v>
-      </c>
-      <c r="J10" s="1">
-        <v>46139</v>
-      </c>
-      <c r="K10">
-        <v>-99</v>
-      </c>
-      <c r="L10" t="s">
-        <v>33</v>
-      </c>
-      <c r="M10" t="s">
-        <v>36</v>
       </c>
     </row>
     <row r="11" spans="1:13" x14ac:dyDescent="0.5">
       <c r="A11" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="B11" t="s">
+        <v>36</v>
+      </c>
+      <c r="C11">
+        <v>5</v>
+      </c>
+      <c r="D11">
+        <v>4</v>
+      </c>
+      <c r="E11">
+        <v>1</v>
+      </c>
+      <c r="F11">
+        <v>0</v>
+      </c>
+      <c r="H11">
+        <v>0</v>
+      </c>
+      <c r="I11">
+        <v>0</v>
+      </c>
+      <c r="J11" s="1">
+        <v>46226</v>
+      </c>
+      <c r="K11">
+        <v>-32</v>
+      </c>
+      <c r="L11" t="s">
         <v>37</v>
-      </c>
-      <c r="C11">
-        <v>35</v>
-      </c>
-      <c r="D11">
-        <v>0</v>
-      </c>
-      <c r="E11">
-        <v>20</v>
-      </c>
-      <c r="F11">
-        <v>0</v>
-      </c>
-      <c r="H11">
-        <v>15</v>
-      </c>
-      <c r="I11">
-        <v>0</v>
-      </c>
-      <c r="J11" s="1">
-        <v>46155</v>
-      </c>
-      <c r="K11">
-        <v>-83</v>
-      </c>
-      <c r="L11" t="s">
-        <v>38</v>
-      </c>
-      <c r="M11" t="s">
-        <v>39</v>
       </c>
     </row>
     <row r="12" spans="1:13" x14ac:dyDescent="0.5">
       <c r="A12" t="s">
+        <v>38</v>
+      </c>
+      <c r="B12" t="s">
+        <v>39</v>
+      </c>
+      <c r="C12">
+        <v>34</v>
+      </c>
+      <c r="D12">
+        <v>0</v>
+      </c>
+      <c r="E12">
+        <v>1</v>
+      </c>
+      <c r="F12">
+        <v>0</v>
+      </c>
+      <c r="H12">
+        <v>15</v>
+      </c>
+      <c r="I12">
+        <v>18</v>
+      </c>
+      <c r="J12" s="1">
+        <v>46231</v>
+      </c>
+      <c r="K12">
+        <v>-27</v>
+      </c>
+      <c r="L12" t="s">
         <v>40</v>
-      </c>
-      <c r="B12" t="s">
-        <v>41</v>
-      </c>
-      <c r="C12">
-        <v>1</v>
-      </c>
-      <c r="D12">
-        <v>0</v>
-      </c>
-      <c r="E12">
-        <v>1</v>
-      </c>
-      <c r="F12">
-        <v>0</v>
-      </c>
-      <c r="H12">
-        <v>0</v>
-      </c>
-      <c r="I12">
-        <v>0</v>
-      </c>
-      <c r="J12" s="1">
-        <v>46188</v>
-      </c>
-      <c r="K12">
-        <v>-50</v>
-      </c>
-      <c r="L12" t="s">
-        <v>42</v>
       </c>
     </row>
     <row r="13" spans="1:13" x14ac:dyDescent="0.5">
       <c r="A13" t="s">
-        <v>43</v>
+        <v>26</v>
       </c>
       <c r="B13" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="C13">
-        <v>5</v>
+        <v>21</v>
       </c>
       <c r="D13">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="E13">
         <v>1</v>
@@ -1411,71 +1399,71 @@
         <v>0</v>
       </c>
       <c r="H13">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="I13">
         <v>0</v>
       </c>
       <c r="J13" s="1">
-        <v>46226</v>
+        <v>46275</v>
       </c>
       <c r="K13">
-        <v>-12</v>
+        <v>17</v>
       </c>
       <c r="L13" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
     </row>
     <row r="14" spans="1:13" x14ac:dyDescent="0.5">
       <c r="A14" t="s">
-        <v>46</v>
+        <v>43</v>
       </c>
       <c r="B14" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="C14">
-        <v>34</v>
+        <v>694</v>
       </c>
       <c r="D14">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E14">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F14">
-        <v>0</v>
+        <v>28</v>
       </c>
       <c r="H14">
-        <v>29</v>
+        <v>663</v>
       </c>
       <c r="I14">
         <v>0</v>
       </c>
       <c r="J14" s="1">
-        <v>46231</v>
+        <v>46261</v>
       </c>
       <c r="K14">
-        <v>-7</v>
+        <v>3</v>
       </c>
       <c r="L14" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
     </row>
     <row r="15" spans="1:13" x14ac:dyDescent="0.5">
       <c r="A15" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="B15" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="C15">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="D15">
         <v>0</v>
       </c>
       <c r="E15">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F15">
         <v>0</v>
@@ -1484,33 +1472,33 @@
         <v>0</v>
       </c>
       <c r="I15">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="J15" s="1">
-        <v>46232</v>
+        <v>46260</v>
       </c>
       <c r="K15">
-        <v>-6</v>
+        <v>2</v>
       </c>
       <c r="L15" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
     </row>
     <row r="16" spans="1:13" x14ac:dyDescent="0.5">
       <c r="A16" t="s">
-        <v>31</v>
+        <v>46</v>
       </c>
       <c r="B16" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="C16">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="D16">
         <v>0</v>
       </c>
       <c r="E16">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F16">
         <v>0</v>
@@ -1522,91 +1510,91 @@
         <v>0</v>
       </c>
       <c r="J16" s="1">
-        <v>46252</v>
+        <v>46260</v>
       </c>
       <c r="K16">
-        <v>14</v>
+        <v>2</v>
       </c>
       <c r="L16" t="s">
-        <v>53</v>
+        <v>48</v>
       </c>
     </row>
     <row r="17" spans="1:12" x14ac:dyDescent="0.5">
       <c r="A17" t="s">
-        <v>54</v>
+        <v>50</v>
       </c>
       <c r="B17" t="s">
-        <v>55</v>
+        <v>51</v>
       </c>
       <c r="C17">
-        <v>55</v>
+        <v>184</v>
       </c>
       <c r="D17">
         <v>0</v>
       </c>
       <c r="E17">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="F17">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="H17">
-        <v>47</v>
+        <v>182</v>
       </c>
       <c r="I17">
         <v>0</v>
       </c>
       <c r="J17" s="1">
-        <v>46247</v>
+        <v>46259</v>
       </c>
       <c r="K17">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="L17" t="s">
-        <v>56</v>
+        <v>52</v>
       </c>
     </row>
     <row r="18" spans="1:12" x14ac:dyDescent="0.5">
       <c r="A18" t="s">
-        <v>57</v>
+        <v>53</v>
       </c>
       <c r="B18" t="s">
-        <v>58</v>
+        <v>54</v>
       </c>
       <c r="C18">
-        <v>59</v>
+        <v>55</v>
       </c>
       <c r="D18">
         <v>0</v>
       </c>
       <c r="E18">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="F18">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H18">
-        <v>56</v>
+        <v>51</v>
       </c>
       <c r="I18">
         <v>0</v>
       </c>
       <c r="J18" s="1">
-        <v>46244</v>
+        <v>46258</v>
       </c>
       <c r="K18">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="L18" t="s">
-        <v>59</v>
+        <v>55</v>
       </c>
     </row>
     <row r="19" spans="1:12" x14ac:dyDescent="0.5">
       <c r="A19" t="s">
-        <v>60</v>
+        <v>56</v>
       </c>
       <c r="B19" t="s">
-        <v>61</v>
+        <v>57</v>
       </c>
       <c r="C19">
         <v>50</v>
@@ -1629,13 +1617,13 @@
     </row>
     <row r="20" spans="1:12" x14ac:dyDescent="0.5">
       <c r="A20" t="s">
-        <v>57</v>
+        <v>46</v>
       </c>
       <c r="B20" t="s">
-        <v>62</v>
+        <v>58</v>
       </c>
       <c r="C20">
-        <v>10</v>
+        <v>66</v>
       </c>
       <c r="D20">
         <v>0</v>
@@ -1644,10 +1632,10 @@
         <v>0</v>
       </c>
       <c r="F20">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="H20">
-        <v>0</v>
+        <v>58</v>
       </c>
       <c r="I20">
         <v>0</v>
@@ -1655,25 +1643,25 @@
     </row>
     <row r="21" spans="1:12" x14ac:dyDescent="0.5">
       <c r="A21" t="s">
-        <v>63</v>
+        <v>59</v>
       </c>
       <c r="B21" t="s">
-        <v>64</v>
+        <v>60</v>
       </c>
       <c r="C21">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="D21">
         <v>0</v>
       </c>
       <c r="E21">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="F21">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="H21">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="I21">
         <v>0</v>
@@ -1681,13 +1669,13 @@
     </row>
     <row r="22" spans="1:12" x14ac:dyDescent="0.5">
       <c r="A22" t="s">
-        <v>57</v>
+        <v>35</v>
       </c>
       <c r="B22" t="s">
-        <v>65</v>
+        <v>61</v>
       </c>
       <c r="C22">
-        <v>5</v>
+        <v>18</v>
       </c>
       <c r="D22">
         <v>0</v>
@@ -1696,10 +1684,10 @@
         <v>0</v>
       </c>
       <c r="F22">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="H22">
-        <v>0</v>
+        <v>15</v>
       </c>
       <c r="I22">
         <v>0</v>
@@ -1707,13 +1695,13 @@
     </row>
     <row r="23" spans="1:12" x14ac:dyDescent="0.5">
       <c r="A23" t="s">
-        <v>43</v>
+        <v>62</v>
       </c>
       <c r="B23" t="s">
-        <v>66</v>
+        <v>63</v>
       </c>
       <c r="C23">
-        <v>17</v>
+        <v>23</v>
       </c>
       <c r="D23">
         <v>0</v>
@@ -1725,7 +1713,7 @@
         <v>2</v>
       </c>
       <c r="H23">
-        <v>15</v>
+        <v>21</v>
       </c>
       <c r="I23">
         <v>0</v>
@@ -1733,10 +1721,10 @@
     </row>
     <row r="24" spans="1:12" x14ac:dyDescent="0.5">
       <c r="A24" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
       <c r="B24" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="C24">
         <v>54</v>
@@ -1759,10 +1747,10 @@
     </row>
     <row r="25" spans="1:12" x14ac:dyDescent="0.5">
       <c r="A25" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="B25" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="C25">
         <v>2</v>
@@ -1785,80 +1773,77 @@
     </row>
     <row r="26" spans="1:12" x14ac:dyDescent="0.5">
       <c r="A26" t="s">
-        <v>71</v>
+        <v>68</v>
       </c>
       <c r="B26" t="s">
-        <v>72</v>
+        <v>69</v>
       </c>
       <c r="C26">
-        <v>16</v>
+        <v>27</v>
       </c>
       <c r="D26">
-        <v>14</v>
+        <v>0</v>
       </c>
       <c r="E26">
         <v>0</v>
       </c>
       <c r="F26">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H26">
-        <v>0</v>
+        <v>18</v>
       </c>
       <c r="I26">
-        <v>0</v>
+        <v>8</v>
       </c>
     </row>
     <row r="27" spans="1:12" x14ac:dyDescent="0.5">
       <c r="A27" t="s">
-        <v>73</v>
+        <v>70</v>
       </c>
       <c r="B27" t="s">
-        <v>74</v>
+        <v>71</v>
       </c>
       <c r="C27">
-        <v>70</v>
+        <v>16</v>
       </c>
       <c r="D27">
         <v>0</v>
       </c>
       <c r="E27">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="F27">
         <v>0</v>
       </c>
       <c r="H27">
-        <v>66</v>
+        <v>0</v>
       </c>
       <c r="I27">
-        <v>0</v>
+        <v>14</v>
       </c>
     </row>
     <row r="28" spans="1:12" x14ac:dyDescent="0.5">
       <c r="A28" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="B28" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="C28">
-        <v>172</v>
+        <v>70</v>
       </c>
       <c r="D28">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E28">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="F28">
         <v>0</v>
       </c>
-      <c r="G28" t="s">
-        <v>77</v>
-      </c>
       <c r="H28">
-        <v>171</v>
+        <v>66</v>
       </c>
       <c r="I28">
         <v>0</v>
@@ -1866,10 +1851,10 @@
     </row>
     <row r="29" spans="1:12" x14ac:dyDescent="0.5">
       <c r="A29" t="s">
-        <v>31</v>
+        <v>26</v>
       </c>
       <c r="B29" t="s">
-        <v>78</v>
+        <v>74</v>
       </c>
       <c r="C29">
         <v>19</v>
@@ -1884,7 +1869,7 @@
         <v>0</v>
       </c>
       <c r="G29" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="H29">
         <v>19</v>
@@ -1895,10 +1880,10 @@
     </row>
     <row r="30" spans="1:12" x14ac:dyDescent="0.5">
       <c r="A30" t="s">
-        <v>31</v>
+        <v>26</v>
       </c>
       <c r="B30" t="s">
-        <v>79</v>
+        <v>76</v>
       </c>
       <c r="C30">
         <v>30</v>
@@ -1913,7 +1898,7 @@
         <v>0</v>
       </c>
       <c r="G30" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="H30">
         <v>30</v>
@@ -1924,10 +1909,10 @@
     </row>
     <row r="31" spans="1:12" x14ac:dyDescent="0.5">
       <c r="A31" t="s">
-        <v>31</v>
+        <v>26</v>
       </c>
       <c r="B31" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
       <c r="C31">
         <v>1</v>
@@ -1942,7 +1927,7 @@
         <v>0</v>
       </c>
       <c r="G31" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="H31">
         <v>1</v>
@@ -1953,10 +1938,10 @@
     </row>
     <row r="32" spans="1:12" x14ac:dyDescent="0.5">
       <c r="A32" t="s">
-        <v>31</v>
+        <v>26</v>
       </c>
       <c r="B32" t="s">
-        <v>81</v>
+        <v>78</v>
       </c>
       <c r="C32">
         <v>1</v>
@@ -1971,7 +1956,7 @@
         <v>0</v>
       </c>
       <c r="G32" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="H32">
         <v>1</v>
@@ -1982,10 +1967,10 @@
     </row>
     <row r="33" spans="1:9" x14ac:dyDescent="0.5">
       <c r="A33" t="s">
-        <v>31</v>
+        <v>26</v>
       </c>
       <c r="B33" t="s">
-        <v>82</v>
+        <v>79</v>
       </c>
       <c r="C33">
         <v>1</v>
@@ -2000,7 +1985,7 @@
         <v>0</v>
       </c>
       <c r="G33" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="H33">
         <v>1</v>
@@ -2011,10 +1996,10 @@
     </row>
     <row r="34" spans="1:9" x14ac:dyDescent="0.5">
       <c r="A34" t="s">
-        <v>31</v>
+        <v>26</v>
       </c>
       <c r="B34" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="C34">
         <v>1</v>
@@ -2029,7 +2014,7 @@
         <v>0</v>
       </c>
       <c r="G34" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="H34">
         <v>1</v>
@@ -2040,10 +2025,10 @@
     </row>
     <row r="35" spans="1:9" x14ac:dyDescent="0.5">
       <c r="A35" t="s">
-        <v>31</v>
+        <v>26</v>
       </c>
       <c r="B35" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
       <c r="C35">
         <v>1</v>
@@ -2058,7 +2043,7 @@
         <v>0</v>
       </c>
       <c r="G35" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="H35">
         <v>1</v>
@@ -2069,10 +2054,10 @@
     </row>
     <row r="36" spans="1:9" x14ac:dyDescent="0.5">
       <c r="A36" t="s">
-        <v>31</v>
+        <v>26</v>
       </c>
       <c r="B36" t="s">
-        <v>85</v>
+        <v>82</v>
       </c>
       <c r="C36">
         <v>1</v>
@@ -2087,7 +2072,7 @@
         <v>0</v>
       </c>
       <c r="G36" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="H36">
         <v>1</v>
@@ -2098,10 +2083,10 @@
     </row>
     <row r="37" spans="1:9" x14ac:dyDescent="0.5">
       <c r="A37" t="s">
-        <v>31</v>
+        <v>26</v>
       </c>
       <c r="B37" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
       <c r="C37">
         <v>6</v>
@@ -2116,7 +2101,7 @@
         <v>0</v>
       </c>
       <c r="G37" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="H37">
         <v>6</v>
@@ -2127,10 +2112,10 @@
     </row>
     <row r="38" spans="1:9" x14ac:dyDescent="0.5">
       <c r="A38" t="s">
-        <v>31</v>
+        <v>26</v>
       </c>
       <c r="B38" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="C38">
         <v>2</v>
@@ -2145,7 +2130,7 @@
         <v>0</v>
       </c>
       <c r="G38" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="H38">
         <v>2</v>
@@ -2156,10 +2141,10 @@
     </row>
     <row r="39" spans="1:9" x14ac:dyDescent="0.5">
       <c r="A39" t="s">
-        <v>31</v>
+        <v>26</v>
       </c>
       <c r="B39" t="s">
-        <v>88</v>
+        <v>85</v>
       </c>
       <c r="C39">
         <v>1</v>
@@ -2174,7 +2159,7 @@
         <v>0</v>
       </c>
       <c r="G39" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="H39">
         <v>1</v>
@@ -2185,10 +2170,10 @@
     </row>
     <row r="40" spans="1:9" x14ac:dyDescent="0.5">
       <c r="A40" t="s">
-        <v>31</v>
+        <v>26</v>
       </c>
       <c r="B40" t="s">
-        <v>89</v>
+        <v>86</v>
       </c>
       <c r="C40">
         <v>4</v>
@@ -2203,7 +2188,7 @@
         <v>0</v>
       </c>
       <c r="G40" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="H40">
         <v>4</v>
@@ -2214,10 +2199,10 @@
     </row>
     <row r="41" spans="1:9" x14ac:dyDescent="0.5">
       <c r="A41" t="s">
-        <v>31</v>
+        <v>26</v>
       </c>
       <c r="B41" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
       <c r="C41">
         <v>1</v>
@@ -2232,7 +2217,7 @@
         <v>0</v>
       </c>
       <c r="G41" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="H41">
         <v>1</v>
@@ -2243,10 +2228,10 @@
     </row>
     <row r="42" spans="1:9" x14ac:dyDescent="0.5">
       <c r="A42" t="s">
-        <v>31</v>
+        <v>26</v>
       </c>
       <c r="B42" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="C42">
         <v>2</v>
@@ -2261,7 +2246,7 @@
         <v>0</v>
       </c>
       <c r="G42" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="H42">
         <v>2</v>
@@ -2272,10 +2257,10 @@
     </row>
     <row r="43" spans="1:9" x14ac:dyDescent="0.5">
       <c r="A43" t="s">
-        <v>31</v>
+        <v>26</v>
       </c>
       <c r="B43" t="s">
-        <v>92</v>
+        <v>89</v>
       </c>
       <c r="C43">
         <v>1</v>
@@ -2290,7 +2275,7 @@
         <v>0</v>
       </c>
       <c r="G43" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="H43">
         <v>1</v>
@@ -2301,10 +2286,10 @@
     </row>
     <row r="44" spans="1:9" x14ac:dyDescent="0.5">
       <c r="A44" t="s">
-        <v>31</v>
+        <v>26</v>
       </c>
       <c r="B44" t="s">
-        <v>93</v>
+        <v>90</v>
       </c>
       <c r="C44">
         <v>9</v>
@@ -2319,7 +2304,7 @@
         <v>0</v>
       </c>
       <c r="G44" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="H44">
         <v>9</v>
@@ -2330,10 +2315,10 @@
     </row>
     <row r="45" spans="1:9" x14ac:dyDescent="0.5">
       <c r="A45" t="s">
-        <v>31</v>
+        <v>26</v>
       </c>
       <c r="B45" t="s">
-        <v>94</v>
+        <v>91</v>
       </c>
       <c r="C45">
         <v>4</v>
@@ -2348,7 +2333,7 @@
         <v>0</v>
       </c>
       <c r="G45" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="H45">
         <v>4</v>
@@ -2359,13 +2344,13 @@
     </row>
     <row r="46" spans="1:9" x14ac:dyDescent="0.5">
       <c r="A46" t="s">
-        <v>31</v>
+        <v>26</v>
       </c>
       <c r="B46" t="s">
-        <v>95</v>
+        <v>92</v>
       </c>
       <c r="C46">
-        <v>20</v>
+        <v>5</v>
       </c>
       <c r="D46">
         <v>0</v>
@@ -2377,10 +2362,10 @@
         <v>0</v>
       </c>
       <c r="G46" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="H46">
-        <v>20</v>
+        <v>5</v>
       </c>
       <c r="I46">
         <v>0</v>
@@ -2388,13 +2373,13 @@
     </row>
     <row r="47" spans="1:9" x14ac:dyDescent="0.5">
       <c r="A47" t="s">
-        <v>31</v>
+        <v>26</v>
       </c>
       <c r="B47" t="s">
-        <v>96</v>
+        <v>93</v>
       </c>
       <c r="C47">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="D47">
         <v>0</v>
@@ -2406,10 +2391,10 @@
         <v>0</v>
       </c>
       <c r="G47" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="H47">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="I47">
         <v>0</v>
@@ -2417,13 +2402,13 @@
     </row>
     <row r="48" spans="1:9" x14ac:dyDescent="0.5">
       <c r="A48" t="s">
-        <v>31</v>
+        <v>26</v>
       </c>
       <c r="B48" t="s">
-        <v>97</v>
+        <v>94</v>
       </c>
       <c r="C48">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D48">
         <v>0</v>
@@ -2435,10 +2420,10 @@
         <v>0</v>
       </c>
       <c r="G48" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="H48">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="I48">
         <v>0</v>
@@ -2446,10 +2431,10 @@
     </row>
     <row r="49" spans="1:9" x14ac:dyDescent="0.5">
       <c r="A49" t="s">
-        <v>31</v>
+        <v>26</v>
       </c>
       <c r="B49" t="s">
-        <v>98</v>
+        <v>95</v>
       </c>
       <c r="C49">
         <v>4</v>
@@ -2464,7 +2449,7 @@
         <v>0</v>
       </c>
       <c r="G49" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="H49">
         <v>4</v>
@@ -2475,13 +2460,13 @@
     </row>
     <row r="50" spans="1:9" x14ac:dyDescent="0.5">
       <c r="A50" t="s">
-        <v>31</v>
+        <v>26</v>
       </c>
       <c r="B50" t="s">
-        <v>99</v>
+        <v>96</v>
       </c>
       <c r="C50">
-        <v>4</v>
+        <v>17</v>
       </c>
       <c r="D50">
         <v>0</v>
@@ -2493,10 +2478,10 @@
         <v>0</v>
       </c>
       <c r="G50" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="H50">
-        <v>4</v>
+        <v>17</v>
       </c>
       <c r="I50">
         <v>0</v>
@@ -2504,13 +2489,13 @@
     </row>
     <row r="51" spans="1:9" x14ac:dyDescent="0.5">
       <c r="A51" t="s">
-        <v>31</v>
+        <v>26</v>
       </c>
       <c r="B51" t="s">
-        <v>100</v>
+        <v>97</v>
       </c>
       <c r="C51">
-        <v>17</v>
+        <v>1</v>
       </c>
       <c r="D51">
         <v>0</v>
@@ -2522,10 +2507,10 @@
         <v>0</v>
       </c>
       <c r="G51" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="H51">
-        <v>17</v>
+        <v>1</v>
       </c>
       <c r="I51">
         <v>0</v>
@@ -2533,10 +2518,10 @@
     </row>
     <row r="52" spans="1:9" x14ac:dyDescent="0.5">
       <c r="A52" t="s">
-        <v>31</v>
+        <v>26</v>
       </c>
       <c r="B52" t="s">
-        <v>101</v>
+        <v>98</v>
       </c>
       <c r="C52">
         <v>1</v>
@@ -2551,7 +2536,7 @@
         <v>0</v>
       </c>
       <c r="G52" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="H52">
         <v>1</v>
@@ -2562,10 +2547,10 @@
     </row>
     <row r="53" spans="1:9" x14ac:dyDescent="0.5">
       <c r="A53" t="s">
-        <v>31</v>
+        <v>26</v>
       </c>
       <c r="B53" t="s">
-        <v>102</v>
+        <v>99</v>
       </c>
       <c r="C53">
         <v>1</v>
@@ -2580,7 +2565,7 @@
         <v>0</v>
       </c>
       <c r="G53" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="H53">
         <v>1</v>
@@ -2591,13 +2576,13 @@
     </row>
     <row r="54" spans="1:9" x14ac:dyDescent="0.5">
       <c r="A54" t="s">
-        <v>31</v>
+        <v>26</v>
       </c>
       <c r="B54" t="s">
-        <v>103</v>
+        <v>100</v>
       </c>
       <c r="C54">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D54">
         <v>0</v>
@@ -2609,10 +2594,10 @@
         <v>0</v>
       </c>
       <c r="G54" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="H54">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="I54">
         <v>0</v>
@@ -2620,13 +2605,13 @@
     </row>
     <row r="55" spans="1:9" x14ac:dyDescent="0.5">
       <c r="A55" t="s">
-        <v>31</v>
+        <v>26</v>
       </c>
       <c r="B55" t="s">
-        <v>104</v>
+        <v>101</v>
       </c>
       <c r="C55">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D55">
         <v>0</v>
@@ -2638,10 +2623,10 @@
         <v>0</v>
       </c>
       <c r="G55" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="H55">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="I55">
         <v>0</v>
@@ -2649,13 +2634,13 @@
     </row>
     <row r="56" spans="1:9" x14ac:dyDescent="0.5">
       <c r="A56" t="s">
-        <v>31</v>
+        <v>26</v>
       </c>
       <c r="B56" t="s">
-        <v>105</v>
+        <v>102</v>
       </c>
       <c r="C56">
-        <v>13</v>
+        <v>20</v>
       </c>
       <c r="D56">
         <v>0</v>
@@ -2667,10 +2652,10 @@
         <v>0</v>
       </c>
       <c r="G56" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="H56">
-        <v>13</v>
+        <v>20</v>
       </c>
       <c r="I56">
         <v>0</v>
@@ -2678,13 +2663,13 @@
     </row>
     <row r="57" spans="1:9" x14ac:dyDescent="0.5">
       <c r="A57" t="s">
-        <v>31</v>
+        <v>26</v>
       </c>
       <c r="B57" t="s">
-        <v>106</v>
+        <v>103</v>
       </c>
       <c r="C57">
-        <v>1</v>
+        <v>13</v>
       </c>
       <c r="D57">
         <v>0</v>
@@ -2696,10 +2681,10 @@
         <v>0</v>
       </c>
       <c r="G57" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="H57">
-        <v>1</v>
+        <v>13</v>
       </c>
       <c r="I57">
         <v>0</v>
@@ -2707,10 +2692,10 @@
     </row>
     <row r="58" spans="1:9" x14ac:dyDescent="0.5">
       <c r="A58" t="s">
-        <v>107</v>
+        <v>26</v>
       </c>
       <c r="B58" t="s">
-        <v>108</v>
+        <v>104</v>
       </c>
       <c r="C58">
         <v>1</v>
@@ -2725,7 +2710,7 @@
         <v>0</v>
       </c>
       <c r="G58" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="H58">
         <v>1</v>
@@ -2736,13 +2721,13 @@
     </row>
     <row r="59" spans="1:9" x14ac:dyDescent="0.5">
       <c r="A59" t="s">
-        <v>109</v>
+        <v>105</v>
       </c>
       <c r="B59" t="s">
-        <v>110</v>
+        <v>106</v>
       </c>
       <c r="C59">
-        <v>33</v>
+        <v>1</v>
       </c>
       <c r="D59">
         <v>0</v>
@@ -2754,10 +2739,10 @@
         <v>0</v>
       </c>
       <c r="G59" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="H59">
-        <v>33</v>
+        <v>1</v>
       </c>
       <c r="I59">
         <v>0</v>
@@ -2765,13 +2750,13 @@
     </row>
     <row r="60" spans="1:9" x14ac:dyDescent="0.5">
       <c r="A60" t="s">
-        <v>111</v>
+        <v>107</v>
       </c>
       <c r="B60" t="s">
-        <v>112</v>
+        <v>108</v>
       </c>
       <c r="C60">
-        <v>50</v>
+        <v>259</v>
       </c>
       <c r="D60">
         <v>0</v>
@@ -2783,10 +2768,10 @@
         <v>0</v>
       </c>
       <c r="G60" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="H60">
-        <v>50</v>
+        <v>259</v>
       </c>
       <c r="I60">
         <v>0</v>
@@ -2794,13 +2779,13 @@
     </row>
     <row r="61" spans="1:9" x14ac:dyDescent="0.5">
       <c r="A61" t="s">
-        <v>49</v>
+        <v>109</v>
       </c>
       <c r="B61" t="s">
-        <v>113</v>
+        <v>110</v>
       </c>
       <c r="C61">
-        <v>1</v>
+        <v>33</v>
       </c>
       <c r="D61">
         <v>0</v>
@@ -2812,10 +2797,10 @@
         <v>0</v>
       </c>
       <c r="G61" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="H61">
-        <v>1</v>
+        <v>33</v>
       </c>
       <c r="I61">
         <v>0</v>
@@ -2823,13 +2808,13 @@
     </row>
     <row r="62" spans="1:9" x14ac:dyDescent="0.5">
       <c r="A62" t="s">
-        <v>49</v>
+        <v>111</v>
       </c>
       <c r="B62" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="C62">
-        <v>2</v>
+        <v>50</v>
       </c>
       <c r="D62">
         <v>0</v>
@@ -2841,10 +2826,10 @@
         <v>0</v>
       </c>
       <c r="G62" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="H62">
-        <v>2</v>
+        <v>50</v>
       </c>
       <c r="I62">
         <v>0</v>
@@ -2852,13 +2837,13 @@
     </row>
     <row r="63" spans="1:9" x14ac:dyDescent="0.5">
       <c r="A63" t="s">
-        <v>49</v>
+        <v>113</v>
       </c>
       <c r="B63" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="C63">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="D63">
         <v>0</v>
@@ -2870,10 +2855,10 @@
         <v>0</v>
       </c>
       <c r="G63" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="H63">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="I63">
         <v>0</v>
@@ -2881,13 +2866,13 @@
     </row>
     <row r="64" spans="1:9" x14ac:dyDescent="0.5">
       <c r="A64" t="s">
-        <v>49</v>
+        <v>113</v>
       </c>
       <c r="B64" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="C64">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D64">
         <v>0</v>
@@ -2899,10 +2884,10 @@
         <v>0</v>
       </c>
       <c r="G64" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="H64">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I64">
         <v>0</v>
@@ -2910,13 +2895,13 @@
     </row>
     <row r="65" spans="1:9" x14ac:dyDescent="0.5">
       <c r="A65" t="s">
-        <v>117</v>
+        <v>113</v>
       </c>
       <c r="B65" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="C65">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="D65">
         <v>0</v>
@@ -2928,10 +2913,10 @@
         <v>0</v>
       </c>
       <c r="G65" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="H65">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="I65">
         <v>0</v>
@@ -2939,13 +2924,13 @@
     </row>
     <row r="66" spans="1:9" x14ac:dyDescent="0.5">
       <c r="A66" t="s">
-        <v>119</v>
+        <v>113</v>
       </c>
       <c r="B66" t="s">
-        <v>120</v>
+        <v>117</v>
       </c>
       <c r="C66">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D66">
         <v>0</v>
@@ -2957,10 +2942,10 @@
         <v>0</v>
       </c>
       <c r="G66" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="H66">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="I66">
         <v>0</v>
@@ -2968,13 +2953,13 @@
     </row>
     <row r="67" spans="1:9" x14ac:dyDescent="0.5">
       <c r="A67" t="s">
-        <v>121</v>
+        <v>113</v>
       </c>
       <c r="B67" t="s">
-        <v>122</v>
+        <v>118</v>
       </c>
       <c r="C67">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D67">
         <v>0</v>
@@ -2986,10 +2971,10 @@
         <v>0</v>
       </c>
       <c r="G67" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="H67">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I67">
         <v>0</v>
@@ -2997,10 +2982,10 @@
     </row>
     <row r="68" spans="1:9" x14ac:dyDescent="0.5">
       <c r="A68" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="B68" t="s">
-        <v>123</v>
+        <v>120</v>
       </c>
       <c r="C68">
         <v>1</v>
@@ -3015,7 +3000,7 @@
         <v>0</v>
       </c>
       <c r="G68" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="H68">
         <v>1</v>
@@ -3026,13 +3011,13 @@
     </row>
     <row r="69" spans="1:9" x14ac:dyDescent="0.5">
       <c r="A69" t="s">
-        <v>124</v>
+        <v>121</v>
       </c>
       <c r="B69" t="s">
-        <v>125</v>
+        <v>122</v>
       </c>
       <c r="C69">
-        <v>30</v>
+        <v>1</v>
       </c>
       <c r="D69">
         <v>0</v>
@@ -3044,10 +3029,10 @@
         <v>0</v>
       </c>
       <c r="G69" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="H69">
-        <v>30</v>
+        <v>1</v>
       </c>
       <c r="I69">
         <v>0</v>
@@ -3055,13 +3040,13 @@
     </row>
     <row r="70" spans="1:9" x14ac:dyDescent="0.5">
       <c r="A70" t="s">
+        <v>123</v>
+      </c>
+      <c r="B70" t="s">
         <v>124</v>
       </c>
-      <c r="B70" t="s">
-        <v>126</v>
-      </c>
       <c r="C70">
-        <v>17</v>
+        <v>2</v>
       </c>
       <c r="D70">
         <v>0</v>
@@ -3073,10 +3058,10 @@
         <v>0</v>
       </c>
       <c r="G70" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="H70">
-        <v>17</v>
+        <v>2</v>
       </c>
       <c r="I70">
         <v>0</v>
@@ -3084,10 +3069,10 @@
     </row>
     <row r="71" spans="1:9" x14ac:dyDescent="0.5">
       <c r="A71" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="B71" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="C71">
         <v>1</v>
@@ -3102,7 +3087,7 @@
         <v>0</v>
       </c>
       <c r="G71" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="H71">
         <v>1</v>
@@ -3113,13 +3098,13 @@
     </row>
     <row r="72" spans="1:9" x14ac:dyDescent="0.5">
       <c r="A72" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="B72" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="C72">
-        <v>2</v>
+        <v>30</v>
       </c>
       <c r="D72">
         <v>0</v>
@@ -3131,10 +3116,10 @@
         <v>0</v>
       </c>
       <c r="G72" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="H72">
-        <v>2</v>
+        <v>30</v>
       </c>
       <c r="I72">
         <v>0</v>
@@ -3142,13 +3127,13 @@
     </row>
     <row r="73" spans="1:9" x14ac:dyDescent="0.5">
       <c r="A73" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="B73" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="C73">
-        <v>10</v>
+        <v>17</v>
       </c>
       <c r="D73">
         <v>0</v>
@@ -3160,10 +3145,10 @@
         <v>0</v>
       </c>
       <c r="G73" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="H73">
-        <v>10</v>
+        <v>17</v>
       </c>
       <c r="I73">
         <v>0</v>
@@ -3171,13 +3156,13 @@
     </row>
     <row r="74" spans="1:9" x14ac:dyDescent="0.5">
       <c r="A74" t="s">
-        <v>130</v>
+        <v>126</v>
       </c>
       <c r="B74" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="C74">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="D74">
         <v>0</v>
@@ -3189,10 +3174,10 @@
         <v>0</v>
       </c>
       <c r="G74" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="H74">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="I74">
         <v>0</v>
@@ -3200,13 +3185,13 @@
     </row>
     <row r="75" spans="1:9" x14ac:dyDescent="0.5">
       <c r="A75" t="s">
+        <v>126</v>
+      </c>
+      <c r="B75" t="s">
         <v>130</v>
       </c>
-      <c r="B75" t="s">
-        <v>132</v>
-      </c>
       <c r="C75">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="D75">
         <v>0</v>
@@ -3218,10 +3203,10 @@
         <v>0</v>
       </c>
       <c r="G75" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="H75">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="I75">
         <v>0</v>
@@ -3229,13 +3214,13 @@
     </row>
     <row r="76" spans="1:9" x14ac:dyDescent="0.5">
       <c r="A76" t="s">
-        <v>133</v>
+        <v>126</v>
       </c>
       <c r="B76" t="s">
-        <v>134</v>
+        <v>131</v>
       </c>
       <c r="C76">
-        <v>19</v>
+        <v>10</v>
       </c>
       <c r="D76">
         <v>0</v>
@@ -3247,10 +3232,10 @@
         <v>0</v>
       </c>
       <c r="G76" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="H76">
-        <v>19</v>
+        <v>10</v>
       </c>
       <c r="I76">
         <v>0</v>
@@ -3258,13 +3243,13 @@
     </row>
     <row r="77" spans="1:9" x14ac:dyDescent="0.5">
       <c r="A77" t="s">
+        <v>132</v>
+      </c>
+      <c r="B77" t="s">
         <v>133</v>
       </c>
-      <c r="B77" t="s">
-        <v>135</v>
-      </c>
       <c r="C77">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="D77">
         <v>0</v>
@@ -3276,10 +3261,10 @@
         <v>0</v>
       </c>
       <c r="G77" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="H77">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="I77">
         <v>0</v>
@@ -3287,13 +3272,13 @@
     </row>
     <row r="78" spans="1:9" x14ac:dyDescent="0.5">
       <c r="A78" t="s">
-        <v>136</v>
+        <v>132</v>
       </c>
       <c r="B78" t="s">
-        <v>137</v>
+        <v>134</v>
       </c>
       <c r="C78">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="D78">
         <v>0</v>
@@ -3305,10 +3290,10 @@
         <v>0</v>
       </c>
       <c r="G78" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="H78">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="I78">
         <v>0</v>
@@ -3316,13 +3301,13 @@
     </row>
     <row r="79" spans="1:9" x14ac:dyDescent="0.5">
       <c r="A79" t="s">
-        <v>138</v>
+        <v>59</v>
       </c>
       <c r="B79" t="s">
-        <v>139</v>
+        <v>135</v>
       </c>
       <c r="C79">
-        <v>28</v>
+        <v>10</v>
       </c>
       <c r="D79">
         <v>0</v>
@@ -3334,10 +3319,10 @@
         <v>0</v>
       </c>
       <c r="G79" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="H79">
-        <v>28</v>
+        <v>10</v>
       </c>
       <c r="I79">
         <v>0</v>
@@ -3345,13 +3330,13 @@
     </row>
     <row r="80" spans="1:9" x14ac:dyDescent="0.5">
       <c r="A80" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="B80" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
       <c r="C80">
-        <v>21</v>
+        <v>2</v>
       </c>
       <c r="D80">
         <v>0</v>
@@ -3363,10 +3348,10 @@
         <v>0</v>
       </c>
       <c r="G80" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="H80">
-        <v>21</v>
+        <v>2</v>
       </c>
       <c r="I80">
         <v>0</v>
@@ -3374,13 +3359,13 @@
     </row>
     <row r="81" spans="1:9" x14ac:dyDescent="0.5">
       <c r="A81" t="s">
+        <v>62</v>
+      </c>
+      <c r="B81" t="s">
         <v>138</v>
       </c>
-      <c r="B81" t="s">
-        <v>141</v>
-      </c>
       <c r="C81">
-        <v>1</v>
+        <v>28</v>
       </c>
       <c r="D81">
         <v>0</v>
@@ -3392,10 +3377,10 @@
         <v>0</v>
       </c>
       <c r="G81" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="H81">
-        <v>1</v>
+        <v>28</v>
       </c>
       <c r="I81">
         <v>0</v>
@@ -3403,13 +3388,13 @@
     </row>
     <row r="82" spans="1:9" x14ac:dyDescent="0.5">
       <c r="A82" t="s">
-        <v>142</v>
+        <v>62</v>
       </c>
       <c r="B82" t="s">
-        <v>143</v>
+        <v>139</v>
       </c>
       <c r="C82">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D82">
         <v>0</v>
@@ -3421,10 +3406,10 @@
         <v>0</v>
       </c>
       <c r="G82" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="H82">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="I82">
         <v>0</v>
@@ -3432,13 +3417,13 @@
     </row>
     <row r="83" spans="1:9" x14ac:dyDescent="0.5">
       <c r="A83" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="B83" t="s">
-        <v>144</v>
+        <v>141</v>
       </c>
       <c r="C83">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D83">
         <v>0</v>
@@ -3450,10 +3435,10 @@
         <v>0</v>
       </c>
       <c r="G83" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="H83">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="I83">
         <v>0</v>
@@ -3461,11 +3446,11 @@
     </row>
     <row r="84" spans="1:9" x14ac:dyDescent="0.5">
       <c r="A84" t="s">
+        <v>140</v>
+      </c>
+      <c r="B84" t="s">
         <v>142</v>
       </c>
-      <c r="B84" t="s">
-        <v>145</v>
-      </c>
       <c r="C84">
         <v>1</v>
       </c>
@@ -3479,7 +3464,7 @@
         <v>0</v>
       </c>
       <c r="G84" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="H84">
         <v>1</v>
@@ -3490,13 +3475,13 @@
     </row>
     <row r="85" spans="1:9" x14ac:dyDescent="0.5">
       <c r="A85" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="B85" t="s">
-        <v>146</v>
+        <v>143</v>
       </c>
       <c r="C85">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D85">
         <v>0</v>
@@ -3508,10 +3493,10 @@
         <v>0</v>
       </c>
       <c r="G85" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="H85">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I85">
         <v>0</v>
@@ -3519,13 +3504,13 @@
     </row>
     <row r="86" spans="1:9" x14ac:dyDescent="0.5">
       <c r="A86" t="s">
-        <v>57</v>
+        <v>140</v>
       </c>
       <c r="B86" t="s">
-        <v>147</v>
+        <v>144</v>
       </c>
       <c r="C86">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D86">
         <v>0</v>
@@ -3537,10 +3522,10 @@
         <v>0</v>
       </c>
       <c r="G86" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="H86">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I86">
         <v>0</v>
@@ -3548,13 +3533,13 @@
     </row>
     <row r="87" spans="1:9" x14ac:dyDescent="0.5">
       <c r="A87" t="s">
-        <v>57</v>
+        <v>46</v>
       </c>
       <c r="B87" t="s">
-        <v>148</v>
+        <v>145</v>
       </c>
       <c r="C87">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D87">
         <v>0</v>
@@ -3566,10 +3551,10 @@
         <v>0</v>
       </c>
       <c r="G87" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="H87">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="I87">
         <v>0</v>
@@ -3577,10 +3562,10 @@
     </row>
     <row r="88" spans="1:9" x14ac:dyDescent="0.5">
       <c r="A88" t="s">
-        <v>57</v>
+        <v>46</v>
       </c>
       <c r="B88" t="s">
-        <v>149</v>
+        <v>146</v>
       </c>
       <c r="C88">
         <v>3</v>
@@ -3595,7 +3580,7 @@
         <v>0</v>
       </c>
       <c r="G88" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="H88">
         <v>3</v>
@@ -3606,10 +3591,10 @@
     </row>
     <row r="89" spans="1:9" x14ac:dyDescent="0.5">
       <c r="A89" t="s">
-        <v>57</v>
+        <v>46</v>
       </c>
       <c r="B89" t="s">
-        <v>150</v>
+        <v>147</v>
       </c>
       <c r="C89">
         <v>3</v>
@@ -3624,7 +3609,7 @@
         <v>0</v>
       </c>
       <c r="G89" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="H89">
         <v>3</v>
@@ -3635,10 +3620,10 @@
     </row>
     <row r="90" spans="1:9" x14ac:dyDescent="0.5">
       <c r="A90" t="s">
-        <v>57</v>
+        <v>46</v>
       </c>
       <c r="B90" t="s">
-        <v>151</v>
+        <v>148</v>
       </c>
       <c r="C90">
         <v>3</v>
@@ -3653,7 +3638,7 @@
         <v>0</v>
       </c>
       <c r="G90" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="H90">
         <v>3</v>
@@ -3664,13 +3649,13 @@
     </row>
     <row r="91" spans="1:9" x14ac:dyDescent="0.5">
       <c r="A91" t="s">
-        <v>57</v>
+        <v>46</v>
       </c>
       <c r="B91" t="s">
-        <v>152</v>
+        <v>149</v>
       </c>
       <c r="C91">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="D91">
         <v>0</v>
@@ -3682,10 +3667,10 @@
         <v>0</v>
       </c>
       <c r="G91" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="H91">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="I91">
         <v>0</v>
@@ -3693,13 +3678,13 @@
     </row>
     <row r="92" spans="1:9" x14ac:dyDescent="0.5">
       <c r="A92" t="s">
-        <v>57</v>
+        <v>46</v>
       </c>
       <c r="B92" t="s">
-        <v>153</v>
+        <v>150</v>
       </c>
       <c r="C92">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="D92">
         <v>0</v>
@@ -3711,10 +3696,10 @@
         <v>0</v>
       </c>
       <c r="G92" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="H92">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="I92">
         <v>0</v>
@@ -3722,13 +3707,13 @@
     </row>
     <row r="93" spans="1:9" x14ac:dyDescent="0.5">
       <c r="A93" t="s">
-        <v>57</v>
+        <v>46</v>
       </c>
       <c r="B93" t="s">
-        <v>154</v>
+        <v>151</v>
       </c>
       <c r="C93">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="D93">
         <v>0</v>
@@ -3740,10 +3725,10 @@
         <v>0</v>
       </c>
       <c r="G93" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="H93">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="I93">
         <v>0</v>
@@ -3751,13 +3736,13 @@
     </row>
     <row r="94" spans="1:9" x14ac:dyDescent="0.5">
       <c r="A94" t="s">
-        <v>155</v>
+        <v>46</v>
       </c>
       <c r="B94" t="s">
-        <v>156</v>
+        <v>152</v>
       </c>
       <c r="C94">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="D94">
         <v>0</v>
@@ -3769,10 +3754,10 @@
         <v>0</v>
       </c>
       <c r="G94" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="H94">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="I94">
         <v>0</v>
@@ -3780,13 +3765,13 @@
     </row>
     <row r="95" spans="1:9" x14ac:dyDescent="0.5">
       <c r="A95" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
       <c r="B95" t="s">
-        <v>157</v>
+        <v>154</v>
       </c>
       <c r="C95">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="D95">
         <v>0</v>
@@ -3798,10 +3783,10 @@
         <v>0</v>
       </c>
       <c r="G95" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="H95">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="I95">
         <v>0</v>
@@ -3809,13 +3794,13 @@
     </row>
     <row r="96" spans="1:9" x14ac:dyDescent="0.5">
       <c r="A96" t="s">
-        <v>158</v>
+        <v>153</v>
       </c>
       <c r="B96" t="s">
-        <v>159</v>
+        <v>155</v>
       </c>
       <c r="C96">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="D96">
         <v>0</v>
@@ -3827,10 +3812,10 @@
         <v>0</v>
       </c>
       <c r="G96" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="H96">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="I96">
         <v>0</v>
@@ -3838,13 +3823,13 @@
     </row>
     <row r="97" spans="1:9" x14ac:dyDescent="0.5">
       <c r="A97" t="s">
-        <v>160</v>
+        <v>156</v>
       </c>
       <c r="B97" t="s">
-        <v>161</v>
+        <v>157</v>
       </c>
       <c r="C97">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="D97">
         <v>0</v>
@@ -3856,10 +3841,10 @@
         <v>0</v>
       </c>
       <c r="G97" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="H97">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="I97">
         <v>0</v>
@@ -3867,13 +3852,13 @@
     </row>
     <row r="98" spans="1:9" x14ac:dyDescent="0.5">
       <c r="A98" t="s">
-        <v>160</v>
+        <v>158</v>
       </c>
       <c r="B98" t="s">
-        <v>162</v>
+        <v>159</v>
       </c>
       <c r="C98">
-        <v>5</v>
+        <v>11</v>
       </c>
       <c r="D98">
         <v>0</v>
@@ -3885,10 +3870,10 @@
         <v>0</v>
       </c>
       <c r="G98" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="H98">
-        <v>5</v>
+        <v>11</v>
       </c>
       <c r="I98">
         <v>0</v>
@@ -3896,13 +3881,13 @@
     </row>
     <row r="99" spans="1:9" x14ac:dyDescent="0.5">
       <c r="A99" t="s">
-        <v>163</v>
+        <v>158</v>
       </c>
       <c r="B99" t="s">
-        <v>164</v>
+        <v>160</v>
       </c>
       <c r="C99">
-        <v>21</v>
+        <v>5</v>
       </c>
       <c r="D99">
         <v>0</v>
@@ -3914,10 +3899,10 @@
         <v>0</v>
       </c>
       <c r="G99" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="H99">
-        <v>21</v>
+        <v>5</v>
       </c>
       <c r="I99">
         <v>0</v>
@@ -3925,13 +3910,13 @@
     </row>
     <row r="100" spans="1:9" x14ac:dyDescent="0.5">
       <c r="A100" t="s">
-        <v>163</v>
+        <v>161</v>
       </c>
       <c r="B100" t="s">
-        <v>165</v>
+        <v>162</v>
       </c>
       <c r="C100">
-        <v>1</v>
+        <v>21</v>
       </c>
       <c r="D100">
         <v>0</v>
@@ -3943,10 +3928,10 @@
         <v>0</v>
       </c>
       <c r="G100" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="H100">
-        <v>1</v>
+        <v>21</v>
       </c>
       <c r="I100">
         <v>0</v>
@@ -3954,11 +3939,11 @@
     </row>
     <row r="101" spans="1:9" x14ac:dyDescent="0.5">
       <c r="A101" t="s">
+        <v>161</v>
+      </c>
+      <c r="B101" t="s">
         <v>163</v>
       </c>
-      <c r="B101" t="s">
-        <v>166</v>
-      </c>
       <c r="C101">
         <v>1</v>
       </c>
@@ -3972,7 +3957,7 @@
         <v>0</v>
       </c>
       <c r="G101" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="H101">
         <v>1</v>
@@ -3983,10 +3968,10 @@
     </row>
     <row r="102" spans="1:9" x14ac:dyDescent="0.5">
       <c r="A102" t="s">
-        <v>163</v>
+        <v>161</v>
       </c>
       <c r="B102" t="s">
-        <v>167</v>
+        <v>164</v>
       </c>
       <c r="C102">
         <v>1</v>
@@ -4001,7 +3986,7 @@
         <v>0</v>
       </c>
       <c r="G102" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="H102">
         <v>1</v>
@@ -4012,10 +3997,10 @@
     </row>
     <row r="103" spans="1:9" x14ac:dyDescent="0.5">
       <c r="A103" t="s">
-        <v>163</v>
+        <v>161</v>
       </c>
       <c r="B103" t="s">
-        <v>168</v>
+        <v>165</v>
       </c>
       <c r="C103">
         <v>1</v>
@@ -4030,7 +4015,7 @@
         <v>0</v>
       </c>
       <c r="G103" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="H103">
         <v>1</v>
@@ -4041,10 +4026,10 @@
     </row>
     <row r="104" spans="1:9" x14ac:dyDescent="0.5">
       <c r="A104" t="s">
-        <v>163</v>
+        <v>161</v>
       </c>
       <c r="B104" t="s">
-        <v>169</v>
+        <v>166</v>
       </c>
       <c r="C104">
         <v>1</v>
@@ -4059,7 +4044,7 @@
         <v>0</v>
       </c>
       <c r="G104" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="H104">
         <v>1</v>
@@ -4070,10 +4055,10 @@
     </row>
     <row r="105" spans="1:9" x14ac:dyDescent="0.5">
       <c r="A105" t="s">
-        <v>163</v>
+        <v>161</v>
       </c>
       <c r="B105" t="s">
-        <v>170</v>
+        <v>167</v>
       </c>
       <c r="C105">
         <v>1</v>
@@ -4088,7 +4073,7 @@
         <v>0</v>
       </c>
       <c r="G105" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="H105">
         <v>1</v>
@@ -4099,10 +4084,10 @@
     </row>
     <row r="106" spans="1:9" x14ac:dyDescent="0.5">
       <c r="A106" t="s">
-        <v>163</v>
+        <v>161</v>
       </c>
       <c r="B106" t="s">
-        <v>171</v>
+        <v>168</v>
       </c>
       <c r="C106">
         <v>1</v>
@@ -4117,7 +4102,7 @@
         <v>0</v>
       </c>
       <c r="G106" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="H106">
         <v>1</v>
@@ -4128,13 +4113,13 @@
     </row>
     <row r="107" spans="1:9" x14ac:dyDescent="0.5">
       <c r="A107" t="s">
-        <v>163</v>
+        <v>161</v>
       </c>
       <c r="B107" t="s">
-        <v>172</v>
+        <v>169</v>
       </c>
       <c r="C107">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D107">
         <v>0</v>
@@ -4146,10 +4131,10 @@
         <v>0</v>
       </c>
       <c r="G107" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="H107">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="I107">
         <v>0</v>
@@ -4157,13 +4142,13 @@
     </row>
     <row r="108" spans="1:9" x14ac:dyDescent="0.5">
       <c r="A108" t="s">
-        <v>163</v>
+        <v>161</v>
       </c>
       <c r="B108" t="s">
-        <v>173</v>
+        <v>170</v>
       </c>
       <c r="C108">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D108">
         <v>0</v>
@@ -4175,10 +4160,10 @@
         <v>0</v>
       </c>
       <c r="G108" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="H108">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="I108">
         <v>0</v>
@@ -4186,13 +4171,13 @@
     </row>
     <row r="109" spans="1:9" x14ac:dyDescent="0.5">
       <c r="A109" t="s">
-        <v>174</v>
+        <v>161</v>
       </c>
       <c r="B109" t="s">
-        <v>175</v>
+        <v>171</v>
       </c>
       <c r="C109">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D109">
         <v>0</v>
@@ -4204,10 +4189,10 @@
         <v>0</v>
       </c>
       <c r="G109" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="H109">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I109">
         <v>0</v>
@@ -4215,10 +4200,10 @@
     </row>
     <row r="110" spans="1:9" x14ac:dyDescent="0.5">
       <c r="A110" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
       <c r="B110" t="s">
-        <v>176</v>
+        <v>173</v>
       </c>
       <c r="C110">
         <v>2</v>
@@ -4233,7 +4218,7 @@
         <v>0</v>
       </c>
       <c r="G110" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="H110">
         <v>2</v>
@@ -4244,13 +4229,13 @@
     </row>
     <row r="111" spans="1:9" x14ac:dyDescent="0.5">
       <c r="A111" t="s">
-        <v>177</v>
+        <v>172</v>
       </c>
       <c r="B111" t="s">
-        <v>178</v>
+        <v>174</v>
       </c>
       <c r="C111">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D111">
         <v>0</v>
@@ -4262,10 +4247,10 @@
         <v>0</v>
       </c>
       <c r="G111" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="H111">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I111">
         <v>0</v>
@@ -4273,10 +4258,10 @@
     </row>
     <row r="112" spans="1:9" x14ac:dyDescent="0.5">
       <c r="A112" t="s">
-        <v>179</v>
+        <v>175</v>
       </c>
       <c r="B112" t="s">
-        <v>180</v>
+        <v>176</v>
       </c>
       <c r="C112">
         <v>1</v>
@@ -4291,7 +4276,7 @@
         <v>0</v>
       </c>
       <c r="G112" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="H112">
         <v>1</v>
@@ -4302,13 +4287,13 @@
     </row>
     <row r="113" spans="1:9" x14ac:dyDescent="0.5">
       <c r="A113" t="s">
-        <v>181</v>
+        <v>177</v>
       </c>
       <c r="B113" t="s">
-        <v>182</v>
+        <v>178</v>
       </c>
       <c r="C113">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="D113">
         <v>0</v>
@@ -4320,10 +4305,10 @@
         <v>0</v>
       </c>
       <c r="G113" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="H113">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="I113">
         <v>0</v>
@@ -4331,13 +4316,13 @@
     </row>
     <row r="114" spans="1:9" x14ac:dyDescent="0.5">
       <c r="A114" t="s">
-        <v>183</v>
+        <v>179</v>
       </c>
       <c r="B114" t="s">
-        <v>184</v>
+        <v>180</v>
       </c>
       <c r="C114">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="D114">
         <v>0</v>
@@ -4349,10 +4334,10 @@
         <v>0</v>
       </c>
       <c r="G114" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="H114">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="I114">
         <v>0</v>
@@ -4360,13 +4345,13 @@
     </row>
     <row r="115" spans="1:9" x14ac:dyDescent="0.5">
       <c r="A115" t="s">
-        <v>185</v>
+        <v>181</v>
       </c>
       <c r="B115" t="s">
-        <v>186</v>
+        <v>182</v>
       </c>
       <c r="C115">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D115">
         <v>0</v>
@@ -4378,10 +4363,10 @@
         <v>0</v>
       </c>
       <c r="G115" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="H115">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I115">
         <v>0</v>
@@ -4389,10 +4374,10 @@
     </row>
     <row r="116" spans="1:9" x14ac:dyDescent="0.5">
       <c r="A116" t="s">
-        <v>185</v>
+        <v>183</v>
       </c>
       <c r="B116" t="s">
-        <v>187</v>
+        <v>184</v>
       </c>
       <c r="C116">
         <v>2</v>
@@ -4407,7 +4392,7 @@
         <v>0</v>
       </c>
       <c r="G116" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="H116">
         <v>2</v>
@@ -4418,13 +4403,13 @@
     </row>
     <row r="117" spans="1:9" x14ac:dyDescent="0.5">
       <c r="A117" t="s">
-        <v>188</v>
+        <v>183</v>
       </c>
       <c r="B117" t="s">
-        <v>189</v>
+        <v>185</v>
       </c>
       <c r="C117">
-        <v>9</v>
+        <v>2</v>
       </c>
       <c r="D117">
         <v>0</v>
@@ -4436,10 +4421,10 @@
         <v>0</v>
       </c>
       <c r="G117" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="H117">
-        <v>9</v>
+        <v>2</v>
       </c>
       <c r="I117">
         <v>0</v>
@@ -4447,13 +4432,13 @@
     </row>
     <row r="118" spans="1:9" x14ac:dyDescent="0.5">
       <c r="A118" t="s">
-        <v>190</v>
+        <v>186</v>
       </c>
       <c r="B118" t="s">
-        <v>191</v>
+        <v>187</v>
       </c>
       <c r="C118">
-        <v>2</v>
+        <v>9</v>
       </c>
       <c r="D118">
         <v>0</v>
@@ -4465,10 +4450,10 @@
         <v>0</v>
       </c>
       <c r="G118" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="H118">
-        <v>2</v>
+        <v>9</v>
       </c>
       <c r="I118">
         <v>0</v>
@@ -4476,13 +4461,13 @@
     </row>
     <row r="119" spans="1:9" x14ac:dyDescent="0.5">
       <c r="A119" t="s">
-        <v>192</v>
+        <v>188</v>
       </c>
       <c r="B119" t="s">
-        <v>193</v>
+        <v>189</v>
       </c>
       <c r="C119">
-        <v>9</v>
+        <v>2</v>
       </c>
       <c r="D119">
         <v>0</v>
@@ -4494,10 +4479,10 @@
         <v>0</v>
       </c>
       <c r="G119" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="H119">
-        <v>9</v>
+        <v>2</v>
       </c>
       <c r="I119">
         <v>0</v>
@@ -4505,13 +4490,13 @@
     </row>
     <row r="120" spans="1:9" x14ac:dyDescent="0.5">
       <c r="A120" t="s">
-        <v>63</v>
+        <v>190</v>
       </c>
       <c r="B120" t="s">
-        <v>194</v>
+        <v>191</v>
       </c>
       <c r="C120">
-        <v>2</v>
+        <v>9</v>
       </c>
       <c r="D120">
         <v>0</v>
@@ -4523,10 +4508,10 @@
         <v>0</v>
       </c>
       <c r="G120" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="H120">
-        <v>2</v>
+        <v>9</v>
       </c>
       <c r="I120">
         <v>0</v>
@@ -4534,13 +4519,13 @@
     </row>
     <row r="121" spans="1:9" x14ac:dyDescent="0.5">
       <c r="A121" t="s">
-        <v>63</v>
+        <v>68</v>
       </c>
       <c r="B121" t="s">
-        <v>195</v>
+        <v>192</v>
       </c>
       <c r="C121">
-        <v>24</v>
+        <v>2</v>
       </c>
       <c r="D121">
         <v>0</v>
@@ -4552,10 +4537,10 @@
         <v>0</v>
       </c>
       <c r="G121" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="H121">
-        <v>24</v>
+        <v>2</v>
       </c>
       <c r="I121">
         <v>0</v>
@@ -4563,13 +4548,13 @@
     </row>
     <row r="122" spans="1:9" x14ac:dyDescent="0.5">
       <c r="A122" t="s">
-        <v>196</v>
+        <v>68</v>
       </c>
       <c r="B122" t="s">
-        <v>197</v>
+        <v>193</v>
       </c>
       <c r="C122">
-        <v>170</v>
+        <v>24</v>
       </c>
       <c r="D122">
         <v>0</v>
@@ -4581,10 +4566,10 @@
         <v>0</v>
       </c>
       <c r="G122" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="H122">
-        <v>170</v>
+        <v>24</v>
       </c>
       <c r="I122">
         <v>0</v>
@@ -4592,13 +4577,13 @@
     </row>
     <row r="123" spans="1:9" x14ac:dyDescent="0.5">
       <c r="A123" t="s">
-        <v>198</v>
+        <v>194</v>
       </c>
       <c r="B123" t="s">
-        <v>199</v>
+        <v>195</v>
       </c>
       <c r="C123">
-        <v>1</v>
+        <v>170</v>
       </c>
       <c r="D123">
         <v>0</v>
@@ -4610,10 +4595,10 @@
         <v>0</v>
       </c>
       <c r="G123" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="H123">
-        <v>1</v>
+        <v>170</v>
       </c>
       <c r="I123">
         <v>0</v>
@@ -4621,10 +4606,10 @@
     </row>
     <row r="124" spans="1:9" x14ac:dyDescent="0.5">
       <c r="A124" t="s">
-        <v>43</v>
+        <v>196</v>
       </c>
       <c r="B124" t="s">
-        <v>200</v>
+        <v>197</v>
       </c>
       <c r="C124">
         <v>1</v>
@@ -4639,7 +4624,7 @@
         <v>0</v>
       </c>
       <c r="G124" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="H124">
         <v>1</v>
@@ -4650,10 +4635,10 @@
     </row>
     <row r="125" spans="1:9" x14ac:dyDescent="0.5">
       <c r="A125" t="s">
-        <v>43</v>
+        <v>35</v>
       </c>
       <c r="B125" t="s">
-        <v>201</v>
+        <v>198</v>
       </c>
       <c r="C125">
         <v>1</v>
@@ -4668,12 +4653,70 @@
         <v>0</v>
       </c>
       <c r="G125" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="H125">
         <v>1</v>
       </c>
       <c r="I125">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="126" spans="1:9" x14ac:dyDescent="0.5">
+      <c r="A126" t="s">
+        <v>35</v>
+      </c>
+      <c r="B126" t="s">
+        <v>199</v>
+      </c>
+      <c r="C126">
+        <v>1</v>
+      </c>
+      <c r="D126">
+        <v>0</v>
+      </c>
+      <c r="E126">
+        <v>0</v>
+      </c>
+      <c r="F126">
+        <v>0</v>
+      </c>
+      <c r="G126" t="s">
+        <v>75</v>
+      </c>
+      <c r="H126">
+        <v>1</v>
+      </c>
+      <c r="I126">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="127" spans="1:9" x14ac:dyDescent="0.5">
+      <c r="A127" t="s">
+        <v>35</v>
+      </c>
+      <c r="B127" t="s">
+        <v>200</v>
+      </c>
+      <c r="C127">
+        <v>1</v>
+      </c>
+      <c r="D127">
+        <v>0</v>
+      </c>
+      <c r="E127">
+        <v>0</v>
+      </c>
+      <c r="F127">
+        <v>0</v>
+      </c>
+      <c r="G127" t="s">
+        <v>75</v>
+      </c>
+      <c r="H127">
+        <v>1</v>
+      </c>
+      <c r="I127">
         <v>0</v>
       </c>
     </row>

</xml_diff>